<commit_message>
added more lowers Rds switches
</commit_message>
<xml_diff>
--- a/Switch Functions/SiC Data Multitrack.xlsx
+++ b/Switch Functions/SiC Data Multitrack.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Switch Functions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jestrin\MIT Dropbox\Julia Estrin\MIT\Research\GE Vernova\Multi-Level-Multi-Track-Optimization\multi-level-multi-track-optimization\Switch Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D07208A-216A-49AB-BF81-F3027BA4E1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB9098D-2B8E-4030-BA4A-CF81AB1D9BA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="59">
   <si>
     <t>Part Number</t>
   </si>
@@ -186,12 +175,42 @@
   </si>
   <si>
     <t>Navitas G3F13M</t>
+  </si>
+  <si>
+    <t>IMCQ120R005M2H</t>
+  </si>
+  <si>
+    <t>IMCQ120R007M2H</t>
+  </si>
+  <si>
+    <t>IMBG120R008M2H</t>
+  </si>
+  <si>
+    <t>IMCQ120R010M2H</t>
+  </si>
+  <si>
+    <t>AIMBG120R010M1</t>
+  </si>
+  <si>
+    <t>IMBG120R012M2H</t>
+  </si>
+  <si>
+    <t>IMBG120R017M2H</t>
+  </si>
+  <si>
+    <t>IMCQ120R017M2H</t>
+  </si>
+  <si>
+    <t>NTBG014N120M3P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -282,7 +301,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -325,6 +344,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -607,31 +638,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AB20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="12" customWidth="1"/>
-    <col min="3" max="3" width="12.90625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.7265625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.6328125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="10.1796875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="14.6328125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.6328125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="13.08984375" style="2" customWidth="1"/>
-    <col min="14" max="14" width="13.81640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.08984375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="8.7265625" style="2"/>
-    <col min="18" max="24" width="8.7265625" style="2"/>
-    <col min="26" max="27" width="8.7265625" style="2"/>
-    <col min="28" max="28" width="11" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5546875" style="2" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" style="2" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="8.109375" style="2" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="8.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -671,7 +711,7 @@
       <c r="M1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="15" t="s">
         <v>5</v>
       </c>
       <c r="O1" s="1" t="s">
@@ -717,7 +757,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>23</v>
       </c>
@@ -742,7 +782,7 @@
       <c r="M2" s="2">
         <v>13.8</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="16">
         <f>297*0.001</f>
         <v>0.29699999999999999</v>
       </c>
@@ -750,7 +790,7 @@
         <v>175</v>
       </c>
       <c r="Q2" s="10">
-        <f t="shared" ref="Q2:Q10" si="0">V2/AB2</f>
+        <f>V2/AB2</f>
         <v>5.5879945429740792</v>
       </c>
       <c r="R2" s="2">
@@ -766,7 +806,7 @@
         <v>10</v>
       </c>
       <c r="V2" s="2">
-        <f t="shared" ref="V2:V10" si="1">U2-T2</f>
+        <f t="shared" ref="V2:V10" si="0">U2-T2</f>
         <v>5.12</v>
       </c>
       <c r="W2" s="2">
@@ -776,18 +816,18 @@
         <v>3.26</v>
       </c>
       <c r="Y2" s="2">
-        <f t="shared" ref="Y2:Y11" si="2">Z2+AA2</f>
+        <f t="shared" ref="Y2:Y11" si="1">Z2+AA2</f>
         <v>8</v>
       </c>
       <c r="AA2" s="2">
         <v>8</v>
       </c>
       <c r="AB2" s="2">
-        <f t="shared" ref="AB2:AB10" si="3">(W2+X2)/(2*Y2)</f>
+        <f t="shared" ref="AB2:AB10" si="2">(W2+X2)/(2*Y2)</f>
         <v>0.91625000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>26</v>
       </c>
@@ -812,7 +852,7 @@
       <c r="M3" s="2">
         <v>9.0500000000000007</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="16">
         <f>262.8*(0.001)</f>
         <v>0.26280000000000003</v>
       </c>
@@ -823,7 +863,7 @@
         <v>15</v>
       </c>
       <c r="Q3" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="Q3:Q10" si="3">V3/AB3</f>
         <v>23.843137254901961</v>
       </c>
       <c r="R3" s="2">
@@ -839,7 +879,7 @@
         <v>11</v>
       </c>
       <c r="V3" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.8</v>
       </c>
       <c r="W3" s="2">
@@ -849,18 +889,18 @@
         <v>3</v>
       </c>
       <c r="Y3" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="AA3" s="2">
         <v>32</v>
       </c>
       <c r="AB3" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.15937499999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>28</v>
       </c>
@@ -885,7 +925,7 @@
       <c r="M4" s="2">
         <v>9</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="16">
         <f>239*(0.001)</f>
         <v>0.23900000000000002</v>
       </c>
@@ -896,7 +936,7 @@
         <v>11</v>
       </c>
       <c r="Q4" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>5.4193333333333324</v>
       </c>
       <c r="R4" s="2">
@@ -912,7 +952,7 @@
         <v>11.6</v>
       </c>
       <c r="V4" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5.5</v>
       </c>
       <c r="W4" s="2">
@@ -922,7 +962,7 @@
         <v>3</v>
       </c>
       <c r="Y4" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.39</v>
       </c>
       <c r="Z4" s="2">
@@ -932,11 +972,11 @@
         <v>6</v>
       </c>
       <c r="AB4" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0148849797023005</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>34</v>
       </c>
@@ -966,7 +1006,7 @@
       <c r="M5" s="4">
         <v>9</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="16">
         <f>239*(0.001)</f>
         <v>0.23900000000000002</v>
       </c>
@@ -977,7 +1017,7 @@
         <v>11</v>
       </c>
       <c r="Q5" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>5.4193333333333324</v>
       </c>
       <c r="R5" s="2">
@@ -993,7 +1033,7 @@
         <v>11.6</v>
       </c>
       <c r="V5" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5.5</v>
       </c>
       <c r="W5" s="2">
@@ -1003,7 +1043,7 @@
         <v>3</v>
       </c>
       <c r="Y5" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.39</v>
       </c>
       <c r="Z5" s="2">
@@ -1013,11 +1053,11 @@
         <v>6</v>
       </c>
       <c r="AB5" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0148849797023005</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>35</v>
       </c>
@@ -1048,7 +1088,7 @@
       <c r="M6" s="2">
         <v>8.93</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="16">
         <f>321*(0.001)</f>
         <v>0.32100000000000001</v>
       </c>
@@ -1059,7 +1099,7 @@
         <v>11</v>
       </c>
       <c r="Q6" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>4.488311688311688</v>
       </c>
       <c r="R6" s="2">
@@ -1075,7 +1115,7 @@
         <v>9</v>
       </c>
       <c r="V6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.7999999999999998</v>
       </c>
       <c r="W6" s="2">
@@ -1085,7 +1125,7 @@
         <v>2.7</v>
       </c>
       <c r="Y6" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>9.6</v>
       </c>
       <c r="Z6" s="2">
@@ -1095,11 +1135,11 @@
         <v>8</v>
       </c>
       <c r="AB6" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.40104166666666669</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>38</v>
       </c>
@@ -1133,7 +1173,7 @@
       <c r="M7" s="2">
         <v>9.0500000000000007</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="16">
         <f>280*(0.001)</f>
         <v>0.28000000000000003</v>
       </c>
@@ -1144,7 +1184,7 @@
         <v>9</v>
       </c>
       <c r="Q7" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6.4495412844036704</v>
       </c>
       <c r="R7" s="2">
@@ -1160,7 +1200,7 @@
         <v>11</v>
       </c>
       <c r="V7" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.625</v>
       </c>
       <c r="W7" s="2">
@@ -1170,7 +1210,7 @@
         <v>2.8</v>
       </c>
       <c r="Y7" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.6</v>
       </c>
       <c r="Z7" s="2">
@@ -1180,11 +1220,11 @@
         <v>2.5</v>
       </c>
       <c r="AB7" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.71710526315789469</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>40</v>
       </c>
@@ -1215,7 +1255,7 @@
       <c r="M8" s="2">
         <v>9.0500000000000007</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="16">
         <f>260*(0.001)</f>
         <v>0.26</v>
       </c>
@@ -1226,7 +1266,7 @@
         <v>10.4</v>
       </c>
       <c r="Q8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>7.8832727272727272</v>
       </c>
       <c r="R8" s="2">
@@ -1242,7 +1282,7 @@
         <v>6.6</v>
       </c>
       <c r="V8" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.26</v>
       </c>
       <c r="W8" s="2">
@@ -1252,7 +1292,7 @@
         <v>3</v>
       </c>
       <c r="Y8" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>13.3</v>
       </c>
       <c r="Z8" s="2">
@@ -1262,11 +1302,11 @@
         <v>3.3</v>
       </c>
       <c r="AB8" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.41353383458646614</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>42</v>
       </c>
@@ -1294,7 +1334,7 @@
       <c r="M9" s="2">
         <v>14.9</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="16">
         <f>327*(0.001)</f>
         <v>0.32700000000000001</v>
       </c>
@@ -1305,7 +1345,7 @@
         <v>3.5</v>
       </c>
       <c r="Q9" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>3.094736842105263</v>
       </c>
       <c r="R9" s="2">
@@ -1321,7 +1361,7 @@
         <v>4</v>
       </c>
       <c r="V9" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.7999999999999998</v>
       </c>
       <c r="W9" s="2">
@@ -1331,7 +1371,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="Y9" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>9.8000000000000007</v>
       </c>
       <c r="Z9" s="2">
@@ -1341,11 +1381,11 @@
         <v>5</v>
       </c>
       <c r="AB9" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.58163265306122447</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>47</v>
       </c>
@@ -1370,7 +1410,7 @@
       <c r="M10" s="2">
         <v>9.0500000000000007</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="16">
         <f>265*(0.001)</f>
         <v>0.26500000000000001</v>
       </c>
@@ -1381,7 +1421,7 @@
         <v>1.8</v>
       </c>
       <c r="Q10" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>3.9679999999999995</v>
       </c>
       <c r="R10" s="2">
@@ -1397,7 +1437,7 @@
         <v>3.8</v>
       </c>
       <c r="V10" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.5499999999999998</v>
       </c>
       <c r="W10" s="2">
@@ -1407,7 +1447,7 @@
         <v>4.5</v>
       </c>
       <c r="Y10" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="Z10" s="2">
@@ -1417,11 +1457,11 @@
         <v>2</v>
       </c>
       <c r="AB10" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.390625</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>49</v>
       </c>
@@ -1446,7 +1486,7 @@
       <c r="M11" s="2">
         <v>8.93</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="16">
         <f>245*(0.001)</f>
         <v>0.245</v>
       </c>
@@ -1472,7 +1512,7 @@
         <v>3.1</v>
       </c>
       <c r="Y11" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>11.3</v>
       </c>
       <c r="Z11" s="2">
@@ -1480,6 +1520,269 @@
       </c>
       <c r="AA11" s="2">
         <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A12" s="8"/>
+      <c r="B12" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" s="2">
+        <v>428</v>
+      </c>
+      <c r="L12" s="2">
+        <v>20.81</v>
+      </c>
+      <c r="M12" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="N12" s="16">
+        <v>1.2E-2</v>
+      </c>
+      <c r="O12" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K13" s="2">
+        <v>287</v>
+      </c>
+      <c r="L13" s="2">
+        <v>20.81</v>
+      </c>
+      <c r="M13" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="N13" s="16">
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="O13" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" s="2">
+        <v>279</v>
+      </c>
+      <c r="L14" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="M14" s="2">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="N14" s="16">
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="O14" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.13</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K15" s="2">
+        <v>214</v>
+      </c>
+      <c r="L15" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="M15" s="2">
+        <v>20.81</v>
+      </c>
+      <c r="N15" s="16">
+        <v>2.35E-2</v>
+      </c>
+      <c r="O15" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.13</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K16" s="2">
+        <v>268</v>
+      </c>
+      <c r="L16">
+        <v>9.36</v>
+      </c>
+      <c r="M16" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N16" s="16">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="O16" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B17" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0.19</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K17" s="2">
+        <v>176</v>
+      </c>
+      <c r="L17">
+        <v>9.36</v>
+      </c>
+      <c r="M17" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N17" s="16">
+        <v>2.8500000000000001E-2</v>
+      </c>
+      <c r="O17" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K18" s="2">
+        <v>126</v>
+      </c>
+      <c r="L18">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="M18" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N18" s="16">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="O18" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B19" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K19">
+        <v>126</v>
+      </c>
+      <c r="L19">
+        <v>20.81</v>
+      </c>
+      <c r="M19">
+        <v>14.9</v>
+      </c>
+      <c r="N19" s="16">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="O19" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B20" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0.23</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K20" s="2">
+        <v>259</v>
+      </c>
+      <c r="L20" s="2">
+        <v>6.15</v>
+      </c>
+      <c r="M20" s="2">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="N20" s="16">
+        <f>2.1*0.014</f>
+        <v>2.9400000000000003E-2</v>
+      </c>
+      <c r="O20" s="2">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -1494,7 +1797,9 @@
     <hyperlink ref="B9" r:id="rId8" xr:uid="{546DB961-E5A1-4530-8964-ED811E06CAF3}"/>
     <hyperlink ref="B10" r:id="rId9" xr:uid="{7CC752DE-D250-418E-ABB1-0BD92E5A0259}"/>
     <hyperlink ref="B11" r:id="rId10" xr:uid="{7BEE2D56-82F7-49C6-8879-C0BE8FD53B67}"/>
+    <hyperlink ref="B12" r:id="rId11" xr:uid="{80502EE4-4A56-4962-9647-85BFE3348831}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update new multitrack data
</commit_message>
<xml_diff>
--- a/Switch Functions/SiC Data Multitrack.xlsx
+++ b/Switch Functions/SiC Data Multitrack.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Switch Functions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Component\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D07208A-216A-49AB-BF81-F3027BA4E1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F1F4E0-458F-4BF7-A3F2-044982D04B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
   <si>
     <t>Part Number</t>
   </si>
@@ -186,6 +186,36 @@
   </si>
   <si>
     <t>Navitas G3F13M</t>
+  </si>
+  <si>
+    <t>IMCQ120R005M2HXUMA1</t>
+  </si>
+  <si>
+    <t>IMCQ120R007M2HXTMA1</t>
+  </si>
+  <si>
+    <t>Infineon CQ120R005</t>
+  </si>
+  <si>
+    <t>IMBG120R008M2HXTMA1</t>
+  </si>
+  <si>
+    <t>Infineon CQ120R007</t>
+  </si>
+  <si>
+    <t>Infineon BG120R008</t>
+  </si>
+  <si>
+    <t>IMCQ120R010M2HXTMA1</t>
+  </si>
+  <si>
+    <t>Infineon CQ120R010</t>
+  </si>
+  <si>
+    <t>AIMBG120R010M1XTMA1</t>
+  </si>
+  <si>
+    <t>Infineon BG120R010</t>
   </si>
 </sst>
 </file>
@@ -323,7 +353,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -607,10 +637,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
     <col min="2" max="2" width="11.90625" style="12" customWidth="1"/>
     <col min="3" max="3" width="12.90625" style="2" customWidth="1"/>
     <col min="4" max="4" width="12.7265625" style="2" customWidth="1"/>
@@ -750,7 +780,7 @@
         <v>175</v>
       </c>
       <c r="Q2" s="10">
-        <f t="shared" ref="Q2:Q10" si="0">V2/AB2</f>
+        <f t="shared" ref="Q2:Q16" si="0">V2/AB2</f>
         <v>5.5879945429740792</v>
       </c>
       <c r="R2" s="2">
@@ -766,7 +796,7 @@
         <v>10</v>
       </c>
       <c r="V2" s="2">
-        <f t="shared" ref="V2:V10" si="1">U2-T2</f>
+        <f t="shared" ref="V2:V12" si="1">U2-T2</f>
         <v>5.12</v>
       </c>
       <c r="W2" s="2">
@@ -776,14 +806,14 @@
         <v>3.26</v>
       </c>
       <c r="Y2" s="2">
-        <f t="shared" ref="Y2:Y11" si="2">Z2+AA2</f>
+        <f t="shared" ref="Y2:Y16" si="2">Z2+AA2</f>
         <v>8</v>
       </c>
       <c r="AA2" s="2">
         <v>8</v>
       </c>
       <c r="AB2" s="2">
-        <f t="shared" ref="AB2:AB10" si="3">(W2+X2)/(2*Y2)</f>
+        <f t="shared" ref="AB2:AB16" si="3">(W2+X2)/(2*Y2)</f>
         <v>0.91625000000000001</v>
       </c>
     </row>
@@ -1482,18 +1512,403 @@
         <v>10</v>
       </c>
     </row>
+    <row r="12" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" s="2">
+        <v>428</v>
+      </c>
+      <c r="L12" s="2">
+        <v>20.81</v>
+      </c>
+      <c r="M12" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="N12" s="2">
+        <f>11.9*(0.001)</f>
+        <v>1.1900000000000001E-2</v>
+      </c>
+      <c r="O12" s="2">
+        <v>175</v>
+      </c>
+      <c r="P12" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="Q12" s="10">
+        <f t="shared" si="0"/>
+        <v>21.666355140186912</v>
+      </c>
+      <c r="R12" s="2">
+        <v>261</v>
+      </c>
+      <c r="S12" s="2">
+        <v>18</v>
+      </c>
+      <c r="T12" s="2">
+        <v>33.4</v>
+      </c>
+      <c r="U12" s="2">
+        <v>57.3</v>
+      </c>
+      <c r="V12" s="2">
+        <f>U12-T12</f>
+        <v>23.9</v>
+      </c>
+      <c r="W12" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="X12" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y12" s="2">
+        <f t="shared" si="2"/>
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="Z12" s="2">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="AA12" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB12" s="2">
+        <f t="shared" si="3"/>
+        <v>1.1030927835051547</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K13" s="2">
+        <v>287</v>
+      </c>
+      <c r="L13" s="2">
+        <v>20.81</v>
+      </c>
+      <c r="M13" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="N13" s="2">
+        <f>17.7*(0.001)</f>
+        <v>1.77E-2</v>
+      </c>
+      <c r="O13" s="2">
+        <v>175</v>
+      </c>
+      <c r="P13" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="Q13" s="10">
+        <f t="shared" si="0"/>
+        <v>22.816363636363633</v>
+      </c>
+      <c r="R13" s="2">
+        <v>197.2</v>
+      </c>
+      <c r="S13" s="2">
+        <v>18</v>
+      </c>
+      <c r="T13" s="2">
+        <v>29</v>
+      </c>
+      <c r="U13" s="2">
+        <v>46.8</v>
+      </c>
+      <c r="V13" s="2">
+        <f>U13-T13</f>
+        <v>17.799999999999997</v>
+      </c>
+      <c r="W13" s="2">
+        <v>6.8</v>
+      </c>
+      <c r="X13" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y13" s="2">
+        <f t="shared" si="2"/>
+        <v>7.05</v>
+      </c>
+      <c r="Z13" s="2">
+        <v>4.75</v>
+      </c>
+      <c r="AA13" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB13" s="2">
+        <f t="shared" si="3"/>
+        <v>0.78014184397163122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" s="2">
+        <v>279</v>
+      </c>
+      <c r="L14" s="2">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="M14" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N14" s="2">
+        <f>18.3*(0.001)</f>
+        <v>1.83E-2</v>
+      </c>
+      <c r="O14" s="2">
+        <v>175</v>
+      </c>
+      <c r="P14" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="Q14" s="10">
+        <f t="shared" si="0"/>
+        <v>14.166355140186917</v>
+      </c>
+      <c r="R14" s="2">
+        <v>195</v>
+      </c>
+      <c r="S14" s="2">
+        <v>18</v>
+      </c>
+      <c r="T14" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="U14" s="2">
+        <v>41</v>
+      </c>
+      <c r="V14" s="2">
+        <f>U14-T14</f>
+        <v>14.3</v>
+      </c>
+      <c r="W14" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="X14" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y14" s="2">
+        <f t="shared" si="2"/>
+        <v>5.3</v>
+      </c>
+      <c r="Z14" s="2">
+        <v>3</v>
+      </c>
+      <c r="AA14" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB14" s="2">
+        <f t="shared" si="3"/>
+        <v>1.0094339622641508</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.13</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K15" s="2">
+        <v>214</v>
+      </c>
+      <c r="L15" s="2">
+        <v>20.81</v>
+      </c>
+      <c r="M15" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="N15" s="2">
+        <f>23.7*(0.001)</f>
+        <v>2.3699999999999999E-2</v>
+      </c>
+      <c r="O15" s="2">
+        <v>175</v>
+      </c>
+      <c r="P15" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="Q15" s="10">
+        <f t="shared" si="0"/>
+        <v>18.58636363636364</v>
+      </c>
+      <c r="R15" s="2">
+        <v>150.1</v>
+      </c>
+      <c r="S15" s="2">
+        <v>18</v>
+      </c>
+      <c r="T15" s="2">
+        <v>22</v>
+      </c>
+      <c r="U15" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="V15" s="2">
+        <f>U15-T15</f>
+        <v>14.100000000000001</v>
+      </c>
+      <c r="W15" s="2">
+        <v>6.8</v>
+      </c>
+      <c r="X15" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y15" s="2">
+        <f t="shared" si="2"/>
+        <v>7.25</v>
+      </c>
+      <c r="Z15" s="2">
+        <v>4.95</v>
+      </c>
+      <c r="AA15" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB15" s="2">
+        <f t="shared" si="3"/>
+        <v>0.75862068965517238</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.13</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K16" s="2">
+        <v>268</v>
+      </c>
+      <c r="L16" s="2">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="M16" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N16" s="2">
+        <f>17.3*(0.001)</f>
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="O16" s="2">
+        <v>175</v>
+      </c>
+      <c r="P16" s="2">
+        <v>17</v>
+      </c>
+      <c r="Q16" s="10">
+        <f t="shared" si="0"/>
+        <v>14.789915966386554</v>
+      </c>
+      <c r="R16" s="2">
+        <v>178</v>
+      </c>
+      <c r="S16" s="2">
+        <v>20</v>
+      </c>
+      <c r="T16" s="2">
+        <v>28</v>
+      </c>
+      <c r="U16" s="2">
+        <v>48</v>
+      </c>
+      <c r="V16" s="2">
+        <f>U16-T16</f>
+        <v>20</v>
+      </c>
+      <c r="W16" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="X16" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="Y16" s="2">
+        <f t="shared" si="2"/>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="Z16" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="AA16" s="2">
+        <v>2</v>
+      </c>
+      <c r="AB16" s="2">
+        <f t="shared" si="3"/>
+        <v>1.3522727272727273</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{8A5BEB82-5995-4FCD-BE33-34F45413EAD1}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{ED0D05AC-8C49-4034-9C3D-B940CFC00CAD}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{BBEBC879-583B-45B4-82C6-7FB87341C452}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{2A777F97-6E48-4ADF-A994-D90C10400081}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{29F8FA21-F41F-4487-8E5B-D1B2BF61DAD8}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{94234AB6-FEA0-4D7E-B69A-E8F941B10E13}"/>
-    <hyperlink ref="B8" r:id="rId7" xr:uid="{81C906B4-A974-43AD-99FB-921D2BE2B59F}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{546DB961-E5A1-4530-8964-ED811E06CAF3}"/>
-    <hyperlink ref="B10" r:id="rId9" xr:uid="{7CC752DE-D250-418E-ABB1-0BD92E5A0259}"/>
-    <hyperlink ref="B11" r:id="rId10" xr:uid="{7BEE2D56-82F7-49C6-8879-C0BE8FD53B67}"/>
+    <hyperlink ref="B11" r:id="rId3" xr:uid="{7BEE2D56-82F7-49C6-8879-C0BE8FD53B67}"/>
+    <hyperlink ref="B10" r:id="rId4" xr:uid="{7CC752DE-D250-418E-ABB1-0BD92E5A0259}"/>
+    <hyperlink ref="B9" r:id="rId5" xr:uid="{546DB961-E5A1-4530-8964-ED811E06CAF3}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{81C906B4-A974-43AD-99FB-921D2BE2B59F}"/>
+    <hyperlink ref="B7" r:id="rId7" xr:uid="{94234AB6-FEA0-4D7E-B69A-E8F941B10E13}"/>
+    <hyperlink ref="B6" r:id="rId8" xr:uid="{29F8FA21-F41F-4487-8E5B-D1B2BF61DAD8}"/>
+    <hyperlink ref="B5" r:id="rId9" xr:uid="{2A777F97-6E48-4ADF-A994-D90C10400081}"/>
+    <hyperlink ref="B4" r:id="rId10" xr:uid="{BBEBC879-583B-45B4-82C6-7FB87341C452}"/>
+    <hyperlink ref="B12" r:id="rId11" xr:uid="{DD087CED-BE96-4C7F-B324-5A9112061F3C}"/>
+    <hyperlink ref="B13" r:id="rId12" xr:uid="{564C5891-5FB4-42CF-8D98-2463E856DE9B}"/>
+    <hyperlink ref="B14" r:id="rId13" xr:uid="{33B19E0A-F57B-4B0B-878A-DD6CE6941333}"/>
+    <hyperlink ref="B15" r:id="rId14" xr:uid="{6E626D2E-C0A2-4609-B6C1-E5DD43EF0ECB}"/>
+    <hyperlink ref="B16" r:id="rId15" xr:uid="{DA76C68C-BD21-4A25-B86C-E3974390854A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update the calculation with jj25 and jj75. Add fullbridge LLC.
</commit_message>
<xml_diff>
--- a/Switch Functions/SiC Data Multitrack.xlsx
+++ b/Switch Functions/SiC Data Multitrack.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Component\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F1F4E0-458F-4BF7-A3F2-044982D04B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1526BEA-7154-4BF2-BF01-BE7CBCE13690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
   <si>
     <t>Part Number</t>
   </si>
@@ -216,6 +216,30 @@
   </si>
   <si>
     <t>Infineon BG120R010</t>
+  </si>
+  <si>
+    <t>IMBG120R012M2HXTMA1</t>
+  </si>
+  <si>
+    <t>Infineon BG120R012</t>
+  </si>
+  <si>
+    <t>SCT012H90G3AG</t>
+  </si>
+  <si>
+    <t>STM SCT012</t>
+  </si>
+  <si>
+    <t>IMBG120R017M2HXTMA1</t>
+  </si>
+  <si>
+    <t>Infineon BG120R017</t>
+  </si>
+  <si>
+    <t>IMCQ120R017M2HXTMA1</t>
+  </si>
+  <si>
+    <t>Infineon CQ120R017</t>
   </si>
 </sst>
 </file>
@@ -245,7 +269,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,6 +291,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -312,7 +342,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -355,6 +385,9 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -637,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.453125" customWidth="1"/>
@@ -780,7 +813,7 @@
         <v>175</v>
       </c>
       <c r="Q2" s="10">
-        <f t="shared" ref="Q2:Q16" si="0">V2/AB2</f>
+        <f t="shared" ref="Q2:Q20" si="0">V2/AB2</f>
         <v>5.5879945429740792</v>
       </c>
       <c r="R2" s="2">
@@ -796,7 +829,7 @@
         <v>10</v>
       </c>
       <c r="V2" s="2">
-        <f t="shared" ref="V2:V12" si="1">U2-T2</f>
+        <f t="shared" ref="V2:V10" si="1">U2-T2</f>
         <v>5.12</v>
       </c>
       <c r="W2" s="2">
@@ -806,14 +839,14 @@
         <v>3.26</v>
       </c>
       <c r="Y2" s="2">
-        <f t="shared" ref="Y2:Y16" si="2">Z2+AA2</f>
+        <f t="shared" ref="Y2:Y20" si="2">Z2+AA2</f>
         <v>8</v>
       </c>
       <c r="AA2" s="2">
         <v>8</v>
       </c>
       <c r="AB2" s="2">
-        <f t="shared" ref="AB2:AB16" si="3">(W2+X2)/(2*Y2)</f>
+        <f t="shared" ref="AB2:AB20" si="3">(W2+X2)/(2*Y2)</f>
         <v>0.91625000000000001</v>
       </c>
     </row>
@@ -1532,7 +1565,7 @@
         <v>428</v>
       </c>
       <c r="L12" s="2">
-        <v>20.81</v>
+        <v>15.3</v>
       </c>
       <c r="M12" s="2">
         <v>14.9</v>
@@ -1564,7 +1597,7 @@
         <v>57.3</v>
       </c>
       <c r="V12" s="2">
-        <f>U12-T12</f>
+        <f t="shared" ref="V12:V20" si="4">U12-T12</f>
         <v>23.9</v>
       </c>
       <c r="W12" s="2">
@@ -1608,7 +1641,7 @@
         <v>287</v>
       </c>
       <c r="L13" s="2">
-        <v>20.81</v>
+        <v>15.3</v>
       </c>
       <c r="M13" s="2">
         <v>14.9</v>
@@ -1640,7 +1673,7 @@
         <v>46.8</v>
       </c>
       <c r="V13" s="2">
-        <f>U13-T13</f>
+        <f t="shared" si="4"/>
         <v>17.799999999999997</v>
       </c>
       <c r="W13" s="2">
@@ -1716,7 +1749,7 @@
         <v>41</v>
       </c>
       <c r="V14" s="2">
-        <f>U14-T14</f>
+        <f t="shared" si="4"/>
         <v>14.3</v>
       </c>
       <c r="W14" s="2">
@@ -1760,7 +1793,7 @@
         <v>214</v>
       </c>
       <c r="L15" s="2">
-        <v>20.81</v>
+        <v>15.3</v>
       </c>
       <c r="M15" s="2">
         <v>14.9</v>
@@ -1792,7 +1825,7 @@
         <v>36.1</v>
       </c>
       <c r="V15" s="2">
-        <f>U15-T15</f>
+        <f t="shared" si="4"/>
         <v>14.100000000000001</v>
       </c>
       <c r="W15" s="2">
@@ -1868,7 +1901,7 @@
         <v>48</v>
       </c>
       <c r="V16" s="2">
-        <f>U16-T16</f>
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="W16" s="2">
@@ -1890,6 +1923,310 @@
       <c r="AB16" s="2">
         <f t="shared" si="3"/>
         <v>1.3522727272727273</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0.19</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K17" s="2">
+        <v>176</v>
+      </c>
+      <c r="L17" s="2">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="M17" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N17" s="2">
+        <f>28.9*(0.001)</f>
+        <v>2.8899999999999999E-2</v>
+      </c>
+      <c r="O17" s="2">
+        <v>175</v>
+      </c>
+      <c r="P17" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="Q17" s="10">
+        <f t="shared" si="0"/>
+        <v>10.951401869158879</v>
+      </c>
+      <c r="R17" s="2">
+        <v>124</v>
+      </c>
+      <c r="S17" s="2">
+        <v>18</v>
+      </c>
+      <c r="T17" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="U17" s="2">
+        <v>26</v>
+      </c>
+      <c r="V17" s="2">
+        <f t="shared" si="4"/>
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="W17" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="X17" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y17" s="2">
+        <f t="shared" si="2"/>
+        <v>6.3</v>
+      </c>
+      <c r="Z17" s="2">
+        <v>4</v>
+      </c>
+      <c r="AA17" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB17" s="2">
+        <f t="shared" si="3"/>
+        <v>0.84920634920634919</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="2">
+        <v>900</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.24</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K18" s="2">
+        <v>244</v>
+      </c>
+      <c r="L18" s="2">
+        <v>10</v>
+      </c>
+      <c r="M18" s="2">
+        <v>8.4</v>
+      </c>
+      <c r="N18" s="2">
+        <f>18.5*(0.001)</f>
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="O18" s="2">
+        <v>175</v>
+      </c>
+      <c r="P18" s="2">
+        <v>47</v>
+      </c>
+      <c r="Q18" s="10">
+        <f t="shared" si="0"/>
+        <v>45.5</v>
+      </c>
+      <c r="R18" s="2">
+        <v>138</v>
+      </c>
+      <c r="S18" s="2">
+        <v>18</v>
+      </c>
+      <c r="T18" s="2">
+        <v>30</v>
+      </c>
+      <c r="U18" s="2">
+        <v>43</v>
+      </c>
+      <c r="V18" s="2">
+        <f t="shared" si="4"/>
+        <v>13</v>
+      </c>
+      <c r="W18" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="X18" s="2">
+        <v>3.1</v>
+      </c>
+      <c r="Y18" s="2">
+        <f t="shared" si="2"/>
+        <v>16.8</v>
+      </c>
+      <c r="Z18" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="AA18" s="2">
+        <v>15</v>
+      </c>
+      <c r="AB18" s="2">
+        <f t="shared" si="3"/>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K19" s="2">
+        <v>126</v>
+      </c>
+      <c r="L19" s="2">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="M19" s="2">
+        <v>9.0500000000000007</v>
+      </c>
+      <c r="N19" s="2">
+        <f>41*(0.001)</f>
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="O19" s="2">
+        <v>175</v>
+      </c>
+      <c r="P19" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="Q19" s="10">
+        <f t="shared" si="0"/>
+        <v>6.6373831775700936</v>
+      </c>
+      <c r="R19" s="2">
+        <v>89</v>
+      </c>
+      <c r="S19" s="2">
+        <v>18</v>
+      </c>
+      <c r="T19" s="2">
+        <v>12.2</v>
+      </c>
+      <c r="U19" s="2">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="V19" s="2">
+        <f t="shared" si="4"/>
+        <v>6.6999999999999993</v>
+      </c>
+      <c r="W19" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="X19" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y19" s="2">
+        <f t="shared" si="2"/>
+        <v>5.3</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>3</v>
+      </c>
+      <c r="AA19" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB19" s="2">
+        <f t="shared" si="3"/>
+        <v>1.0094339622641508</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="2">
+        <v>1200</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K20" s="2">
+        <v>126</v>
+      </c>
+      <c r="L20" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="M20" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="N20" s="2">
+        <f>40.6*(0.001)</f>
+        <v>4.0600000000000004E-2</v>
+      </c>
+      <c r="O20" s="2">
+        <v>175</v>
+      </c>
+      <c r="P20" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q20" s="10">
+        <f t="shared" si="0"/>
+        <v>8.1309090909090873</v>
+      </c>
+      <c r="R20" s="2">
+        <v>91.1</v>
+      </c>
+      <c r="S20" s="2">
+        <v>18</v>
+      </c>
+      <c r="T20" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="U20" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="V20" s="2">
+        <f t="shared" si="4"/>
+        <v>8.5999999999999979</v>
+      </c>
+      <c r="W20" s="2">
+        <v>6.8</v>
+      </c>
+      <c r="X20" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="Y20" s="2">
+        <f t="shared" si="2"/>
+        <v>5.1999999999999993</v>
+      </c>
+      <c r="Z20" s="2">
+        <v>2.9</v>
+      </c>
+      <c r="AA20" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AB20" s="2">
+        <f t="shared" si="3"/>
+        <v>1.0576923076923079</v>
       </c>
     </row>
   </sheetData>
@@ -1909,6 +2246,10 @@
     <hyperlink ref="B14" r:id="rId13" xr:uid="{33B19E0A-F57B-4B0B-878A-DD6CE6941333}"/>
     <hyperlink ref="B15" r:id="rId14" xr:uid="{6E626D2E-C0A2-4609-B6C1-E5DD43EF0ECB}"/>
     <hyperlink ref="B16" r:id="rId15" xr:uid="{DA76C68C-BD21-4A25-B86C-E3974390854A}"/>
+    <hyperlink ref="B17" r:id="rId16" xr:uid="{184E926F-BDFA-47DA-86FD-BA6D45CC286A}"/>
+    <hyperlink ref="B18" r:id="rId17" xr:uid="{47A65654-2B99-4A42-96F5-4E832953679B}"/>
+    <hyperlink ref="B19" r:id="rId18" xr:uid="{3FBB7AF4-524B-4C2F-9210-A760A8F3CFD1}"/>
+    <hyperlink ref="B20" r:id="rId19" xr:uid="{99DCDDEA-6FF8-43BA-96F2-F6A6D786EEB4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update pin area for SiC devices
</commit_message>
<xml_diff>
--- a/Switch Functions/SiC Data Multitrack.xlsx
+++ b/Switch Functions/SiC Data Multitrack.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Component\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1526BEA-7154-4BF2-BF01-BE7CBCE13690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED85B03F-7BF3-421C-B8E1-2A6E6D599BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="69">
   <si>
     <t>Part Number</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t>Infineon CQ120R017</t>
+  </si>
+  <si>
+    <t>Pin_Area [mm2]</t>
   </si>
 </sst>
 </file>
@@ -670,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB20"/>
+  <dimension ref="A1:AC20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.453125" customWidth="1"/>
@@ -692,9 +695,10 @@
     <col min="18" max="24" width="8.7265625" style="2"/>
     <col min="26" max="27" width="8.7265625" style="2"/>
     <col min="28" max="28" width="11" style="2" customWidth="1"/>
+    <col min="29" max="29" width="14.90625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -779,8 +783,11 @@
       <c r="AB1" s="9" t="s">
         <v>19</v>
       </c>
+      <c r="AC1" s="9" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="2" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>23</v>
       </c>
@@ -849,8 +856,12 @@
         <f t="shared" ref="AB2:AB20" si="3">(W2+X2)/(2*Y2)</f>
         <v>0.91625000000000001</v>
       </c>
+      <c r="AC2" s="2">
+        <f>15.85*(18.7-13.8)</f>
+        <v>77.664999999999978</v>
+      </c>
     </row>
-    <row r="3" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
         <v>26</v>
       </c>
@@ -922,8 +933,12 @@
         <f t="shared" si="3"/>
         <v>0.15937499999999999</v>
       </c>
+      <c r="AC3" s="2">
+        <f>9.8*(4.55+0.87)</f>
+        <v>53.116</v>
+      </c>
     </row>
-    <row r="4" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="12" t="s">
         <v>28</v>
       </c>
@@ -998,8 +1013,12 @@
         <f t="shared" si="3"/>
         <v>1.0148849797023005</v>
       </c>
+      <c r="AC4" s="2">
+        <f>9.7*(15.1-9)</f>
+        <v>59.169999999999995</v>
+      </c>
     </row>
-    <row r="5" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>34</v>
       </c>
@@ -1079,8 +1098,12 @@
         <f t="shared" si="3"/>
         <v>1.0148849797023005</v>
       </c>
+      <c r="AC5" s="2">
+        <f>9.7*(15.1-9)</f>
+        <v>59.169999999999995</v>
+      </c>
     </row>
-    <row r="6" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>35</v>
       </c>
@@ -1161,8 +1184,12 @@
         <f t="shared" si="3"/>
         <v>0.40104166666666669</v>
       </c>
+      <c r="AC6" s="2">
+        <f>10.08*(16.4-0.5-8.93)</f>
+        <v>70.257599999999982</v>
+      </c>
     </row>
-    <row r="7" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>38</v>
       </c>
@@ -1246,8 +1273,12 @@
         <f t="shared" si="3"/>
         <v>0.71710526315789469</v>
       </c>
+      <c r="AC7" s="2">
+        <f>9.8*(14.87-9.05)</f>
+        <v>57.035999999999987</v>
+      </c>
     </row>
-    <row r="8" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>40</v>
       </c>
@@ -1328,8 +1359,12 @@
         <f t="shared" si="3"/>
         <v>0.41353383458646614</v>
       </c>
+      <c r="AC8" s="2">
+        <f>9.8*(14.87-9.05)</f>
+        <v>57.035999999999987</v>
+      </c>
     </row>
-    <row r="9" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>42</v>
       </c>
@@ -1407,8 +1442,12 @@
         <f t="shared" si="3"/>
         <v>0.58163265306122447</v>
       </c>
+      <c r="AC9" s="2">
+        <f>14.9*(20.81-15.3)</f>
+        <v>82.098999999999975</v>
+      </c>
     </row>
-    <row r="10" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>47</v>
       </c>
@@ -1483,8 +1522,12 @@
         <f t="shared" si="3"/>
         <v>0.390625</v>
       </c>
+      <c r="AC10" s="2">
+        <f>9.8*(15-9.05)</f>
+        <v>58.309999999999995</v>
+      </c>
     </row>
-    <row r="11" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>49</v>
       </c>
@@ -1544,8 +1587,12 @@
       <c r="AA11" s="2">
         <v>10</v>
       </c>
+      <c r="AC11" s="2">
+        <f>10.08*(15-8.93)</f>
+        <v>61.185600000000001</v>
+      </c>
     </row>
-    <row r="12" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>52</v>
       </c>
@@ -1620,8 +1667,12 @@
         <f t="shared" si="3"/>
         <v>1.1030927835051547</v>
       </c>
+      <c r="AC12" s="2">
+        <f>14.9*(20.81-15.3)</f>
+        <v>82.098999999999975</v>
+      </c>
     </row>
-    <row r="13" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>54</v>
       </c>
@@ -1696,8 +1747,12 @@
         <f t="shared" si="3"/>
         <v>0.78014184397163122</v>
       </c>
+      <c r="AC13" s="2">
+        <f>14.9*(20.81-15.3)</f>
+        <v>82.098999999999975</v>
+      </c>
     </row>
-    <row r="14" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>55</v>
       </c>
@@ -1772,8 +1827,12 @@
         <f t="shared" si="3"/>
         <v>1.0094339622641508</v>
       </c>
+      <c r="AC14" s="2">
+        <f>9.8*(15-9.05)</f>
+        <v>58.309999999999995</v>
+      </c>
     </row>
-    <row r="15" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>57</v>
       </c>
@@ -1848,8 +1907,12 @@
         <f t="shared" si="3"/>
         <v>0.75862068965517238</v>
       </c>
+      <c r="AC15" s="2">
+        <f>14.9*(20.81-15.3)</f>
+        <v>82.098999999999975</v>
+      </c>
     </row>
-    <row r="16" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
         <v>59</v>
       </c>
@@ -1924,8 +1987,12 @@
         <f t="shared" si="3"/>
         <v>1.3522727272727273</v>
       </c>
+      <c r="AC16" s="2">
+        <f>9.8*(15-9.05)</f>
+        <v>58.309999999999995</v>
+      </c>
     </row>
-    <row r="17" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
         <v>61</v>
       </c>
@@ -2000,8 +2067,12 @@
         <f t="shared" si="3"/>
         <v>0.84920634920634919</v>
       </c>
+      <c r="AC17" s="2">
+        <f>9.8*(15-9.05)</f>
+        <v>58.309999999999995</v>
+      </c>
     </row>
-    <row r="18" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
         <v>63</v>
       </c>
@@ -2024,7 +2095,7 @@
         <v>10</v>
       </c>
       <c r="M18" s="2">
-        <v>8.4</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="N18" s="2">
         <f>18.5*(0.001)</f>
@@ -2076,8 +2147,12 @@
         <f t="shared" si="3"/>
         <v>0.2857142857142857</v>
       </c>
+      <c r="AC18" s="2">
+        <f>10*(1.27+4.35)</f>
+        <v>56.199999999999989</v>
+      </c>
     </row>
-    <row r="19" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
         <v>65</v>
       </c>
@@ -2152,8 +2227,12 @@
         <f t="shared" si="3"/>
         <v>1.0094339622641508</v>
       </c>
+      <c r="AC19" s="2">
+        <f>9.8*(15-9.05)</f>
+        <v>58.309999999999995</v>
+      </c>
     </row>
-    <row r="20" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
         <v>67</v>
       </c>
@@ -2227,6 +2306,10 @@
       <c r="AB20" s="2">
         <f t="shared" si="3"/>
         <v>1.0576923076923079</v>
+      </c>
+      <c r="AC20" s="2">
+        <f>14.9*(20.81-15.3)</f>
+        <v>82.098999999999975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>